<commit_message>
Update import workbooks: Marks Baseline, Roster Gender, Testables tab
</commit_message>
<xml_diff>
--- a/Jaguars-Jumps-Home-Data.xlsx
+++ b/Jaguars-Jumps-Home-Data.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Marks" sheetId="1" r:id="rId1"/>
     <sheet name="Schedule" sheetId="2" r:id="rId2"/>
     <sheet name="Notes" sheetId="3" r:id="rId3"/>
+    <sheet name="Testables" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -399,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" customWidth="1"/>
@@ -407,6 +408,7 @@
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="9.83203125" customWidth="1"/>
     <col min="6" max="6" width="42.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,6 +430,9 @@
       <c r="F1" t="str">
         <v>Goal Note</v>
       </c>
+      <c r="G1" t="str">
+        <v>Baseline</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -448,6 +453,9 @@
       <c r="F2" t="str">
         <v>Three-event anchor — stay tall, ride the board.</v>
       </c>
+      <c r="G2" t="str">
+        <v>18'6.5"</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -468,6 +476,9 @@
       <c r="F3" t="str">
         <v>Step phase is where you leave distance — be patient.</v>
       </c>
+      <c r="G3" t="str">
+        <v>34'6"</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -488,6 +499,9 @@
       <c r="F4" t="str">
         <v>Quick, tall plant — attack the bar.</v>
       </c>
+      <c r="G4" t="str">
+        <v>5'2"</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -508,6 +522,9 @@
       <c r="F5" t="str">
         <v>Closest to Juan — hold your penultimate.</v>
       </c>
+      <c r="G5" t="str">
+        <v>18'3"</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -528,6 +545,9 @@
       <c r="F6" t="str">
         <v>New second event — build a smooth, even rhythm.</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -548,6 +568,9 @@
       <c r="F7" t="str">
         <v>Speed's rising fast — convert it on the board.</v>
       </c>
+      <c r="G7" t="str">
+        <v>16'7"</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -568,6 +591,9 @@
       <c r="F8" t="str">
         <v>Hurdle rhythm = great penultimate. One full season.</v>
       </c>
+      <c r="G8" t="str">
+        <v>16'5.5"</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -588,6 +614,9 @@
       <c r="F9" t="str">
         <v>Our TJ project — even, patient phases.</v>
       </c>
+      <c r="G9" t="str">
+        <v>28'3"</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -608,6 +637,9 @@
       <c r="F10" t="str">
         <v>Second event — fast, flat approach.</v>
       </c>
+      <c r="G10" t="str">
+        <v>14'7.5"</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -628,6 +660,9 @@
       <c r="F11" t="str">
         <v>Steady improver — keep stacking inches.</v>
       </c>
+      <c r="G11" t="str">
+        <v>14'1"</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -648,6 +683,9 @@
       <c r="F12" t="str">
         <v>Match your sprint speed at takeoff.</v>
       </c>
+      <c r="G12" t="str">
+        <v>10'9.5"</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -668,6 +706,9 @@
       <c r="F13" t="str">
         <v>Have fun and score in duals.</v>
       </c>
+      <c r="G13" t="str">
+        <v>12'0"</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -688,6 +729,9 @@
       <c r="F14" t="str">
         <v>Your speed = big LJ potential. Two days a week.</v>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -708,6 +752,9 @@
       <c r="F15" t="str">
         <v>Lead girl horizontals — drive the knee up.</v>
       </c>
+      <c r="G15" t="str">
+        <v>13'1.5"</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -728,6 +775,9 @@
       <c r="F16" t="str">
         <v>Lead girl TJ — hold the step phase.</v>
       </c>
+      <c r="G16" t="str">
+        <v>26'9"</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -748,6 +798,9 @@
       <c r="F17" t="str">
         <v>Flop development — attack the bar.</v>
       </c>
+      <c r="G17" t="str">
+        <v>4'4"</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -768,6 +821,9 @@
       <c r="F18" t="str">
         <v>Secondary event — fast and tall.</v>
       </c>
+      <c r="G18" t="str">
+        <v>12'10.5"</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -788,6 +844,9 @@
       <c r="F19" t="str">
         <v>300H rhythm transfers to TJ — girls TJ is wide open.</v>
       </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -808,6 +867,9 @@
       <c r="F20" t="str">
         <v>Board accuracy is THE focus — trust your steps.</v>
       </c>
+      <c r="G20" t="str">
+        <v>12'5"</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -828,6 +890,9 @@
       <c r="F21" t="str">
         <v>Senior leader — steady, repeatable approach.</v>
       </c>
+      <c r="G21" t="str">
+        <v>4'4"</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -848,6 +913,9 @@
       <c r="F22" t="str">
         <v>Youngest returner — improve every single meet.</v>
       </c>
+      <c r="G22" t="str">
+        <v>12'1.5"</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -868,10 +936,13 @@
       <c r="F23" t="str">
         <v>Start TJ now — you are the future anchor.</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1120,4 +1191,91 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Athlete</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Test</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Result</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Date</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Juan Ledesma</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Standing LJ</v>
+      </c>
+      <c r="C2" t="str">
+        <v>9'2"</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2027-01-09</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Pablo Jara</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Standing LJ</v>
+      </c>
+      <c r="C3" t="str">
+        <v>8'9"</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2027-01-09</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Juan Ledesma</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Flying 10</v>
+      </c>
+      <c r="C4" t="str">
+        <v>1.05</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2027-01-09</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Daniela Gamboa</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Medball Back Toss</v>
+      </c>
+      <c r="C5" t="str">
+        <v>28'0"</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2027-01-09</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Practice Plan view + This Block card (16-block season timeline)
</commit_message>
<xml_diff>
--- a/Jaguars-Jumps-Home-Data.xlsx
+++ b/Jaguars-Jumps-Home-Data.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Schedule" sheetId="2" r:id="rId2"/>
     <sheet name="Notes" sheetId="3" r:id="rId3"/>
     <sheet name="Testables" sheetId="4" r:id="rId4"/>
+    <sheet name="Plan" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -1278,4 +1279,363 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F17"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="80.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Phase</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Start</v>
+      </c>
+      <c r="D1" t="str">
+        <v>End</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Theme</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Focus</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Block 1 · Foundation</v>
+      </c>
+      <c r="B2" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-08-03</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Learn how we move.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Install the full warm-up as a teaching circuit · Speed: acceleration posture (wall drills, falling starts, builds) · Power: medball technique, pogo and line hops · Strength: bodyweight circuit</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Block 2 · Acceleration Emphasis</v>
+      </c>
+      <c r="B3" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Push the ground away.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Speed: sled pushes, push-up starts to 20m accels · Power: measured medball throws, standing broad jumps · Strength: lateral lunges, single-leg glute bridges, Nordics</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Block 3 · Speed Mechanics</v>
+      </c>
+      <c r="B4" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Upright and bouncy.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Speed: wicket runs, flying 10s · Power: low hurdle hops, lateral bounds, intro straight-leg bounds · Strength: goblet squat and RDL patterns</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Block 4 · Max Velocity</v>
+      </c>
+      <c r="B5" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Top speed is a skill.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Speed: flying 20s, full recovery, timed · Power: depth landings to low depth jumps, single-leg control · Strength: light sled pulls plus pattern work</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Block 5 · Power Conversion</v>
+      </c>
+      <c r="B6" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-11-13</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Strength becomes spring.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Speed: maintain flys, runway rhythm runs (no jumping) · Power: alternate bounds, single-leg hops, standing LJ into the pit · Strength: jump circuit</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Block 6 · Event Sampler</v>
+      </c>
+      <c r="B7" t="str">
+        <v>General Prep</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-11-16</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-11-27</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Try out the events.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Stations: short-approach LJ, TJ hop-step rhythm, HJ scissors · Pit safety and runway etiquette · Recruiting window: Donyell, Janell, Emmanuel</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Block 7 · Event Fundamentals</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Winter Track</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-12-18</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Takeoff is everything.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Assign events; split beginner vs advanced · Day A: LJ penultimate + short approach, TJ rhythm, HJ curve/scissors · Day B: lift day at teaching loads · Weekly mark logged</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Block 8 · Approach Construction</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Winter Track</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-12-21</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2027-01-01</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Build the runway.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Establish approaches: step counts and start marks · Mid-approach jumping at 60-70% · Break-proofed, every session standalone</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Block 9 · Competition Introduction</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Winter Competition</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2027-01-04</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2027-01-22</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Jump under the lights.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Mon activation lift + bounds · Tue phase drills + speed · Wed free jumping + approach · Thu approach lock-in · Fri shakeout · Sat qualifier · Monday film</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Block 10 · Winter Sharpening</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Winter Competition</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2027-01-25</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2027-02-06</v>
+      </c>
+      <c r="E11" t="str">
+        <v>First peak rehearsal.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Qualifier 1/30 to Winter Champs 2/6 at Arcadia · Taper: cut volume ~40%, hold intensity · Full approaches Mon/Tue only</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Block 11 · Season Launch</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2027-02-08</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2027-02-19</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Open the spring.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Full February lift menu live 2x/week, supersets · Competition simulation Friday · Feb 20 opener</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Block 12 · Early Season Development</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C13" t="str">
+        <v>2027-02-22</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2027-03-13</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Build through the duals.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Duals are practice with officials; volume stays high · One technical priority per athlete per block · Beginners chase legal jumps + board accuracy</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Block 13 · Technical Block II + Spring Break</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2027-03-16</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2027-04-03</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Sharpen the technique.</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Spring Break drilling week (3/22-26): low intensity, high reps, TJ phase ratios · Final heavy strength push ends here</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Block 14 · First Peak</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2027-04-05</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2027-04-17</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Peak for April.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Arcadia 4/9-10 · Raincross 4/10 · IE Champs 4/17 · Volume drops, rest rises; full approaches early-week only · Weightroom to 1 day/week after 4/17</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Block 15 · League Prep</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2027-04-20</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2027-05-01</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Set up for League.</v>
+      </c>
+      <c r="F16" t="str">
+        <v>League Champs 4/29, event assignments for max team points · One hard CNS day, one jump day, rest is rhythm and recovery</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Block 16 · Championship Series</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Spring Season</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2027-05-03</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2027-05-29</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Chase CIF.</v>
+      </c>
+      <c r="F17" t="str">
+        <v>CIF Prelims 5/8 to Finals to Masters to State · Qualifiers stay in taper rhythm · Everyone else flips to a development block</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Part 2: daily session detail (Sessions tab) + version stamp in health check
</commit_message>
<xml_diff>
--- a/Jaguars-Jumps-Home-Data.xlsx
+++ b/Jaguars-Jumps-Home-Data.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Notes" sheetId="3" r:id="rId3"/>
     <sheet name="Testables" sheetId="4" r:id="rId4"/>
     <sheet name="Plan" sheetId="5" r:id="rId5"/>
+    <sheet name="Sessions" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -1638,4 +1639,371 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="9.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="34.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Intensity</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Goal</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Segment</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Sets/Reps</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Rest</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Cue</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Block 1 · Foundation</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>GPP</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Teach</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Learn the warm-up; install acceleration posture.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Warm-Up</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Standard Warm-Up (Scoops to Build-Ups)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>full teaching circuit</v>
+      </c>
+      <c r="J2" t="str">
+        <v>25</v>
+      </c>
+      <c r="K2" t="str">
+        <v>—</v>
+      </c>
+      <c r="L2" t="str">
+        <v>15m out, walk back; even lines no deeper than 6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>Speed</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Wall drills</v>
+      </c>
+      <c r="I3" t="str">
+        <v>3×10s</v>
+      </c>
+      <c r="J3" t="str">
+        <v>8</v>
+      </c>
+      <c r="K3" t="str">
+        <v>full</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Tall posture, push the ground away</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>Speed</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Falling start to 20m build</v>
+      </c>
+      <c r="I4" t="str">
+        <v>3×20m</v>
+      </c>
+      <c r="J4" t="str">
+        <v>9</v>
+      </c>
+      <c r="K4" t="str">
+        <v>full</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Fall, don't sit; gradual rise</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Speed</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Build-up runs</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2×20m</v>
+      </c>
+      <c r="J5" t="str">
+        <v>8</v>
+      </c>
+      <c r="K5" t="str">
+        <v>walk back</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Smooth acceleration to fast</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Power</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Medball chest pass + overhead back toss</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2×6 each</v>
+      </c>
+      <c r="J6" t="str">
+        <v>12</v>
+      </c>
+      <c r="K6" t="str">
+        <v>60s</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Punch through; hips lead the toss</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>Power</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Pogo + line hops</v>
+      </c>
+      <c r="I7" t="str">
+        <v>3×10</v>
+      </c>
+      <c r="J7" t="str">
+        <v>13</v>
+      </c>
+      <c r="K7" t="str">
+        <v>60s</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Stiff ankle, flat-foot contacts</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>Strength</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Bodyweight circuit (squat / lunge / hinge / push / plank)</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2 rounds</v>
+      </c>
+      <c r="J8" t="str">
+        <v>12</v>
+      </c>
+      <c r="K8" t="str">
+        <v>minimal</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Quality reps, control the movement</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>Wrap</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Log a standing long jump</v>
+      </c>
+      <c r="I9" t="str">
+        <v>1 mark</v>
+      </c>
+      <c r="J9" t="str">
+        <v>3</v>
+      </c>
+      <c r="K9" t="str">
+        <v>—</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Season baseline measurable</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add month-grid Team Calendar (Plan tab) + declutter Coach landing (collapsible lists)
</commit_message>
<xml_diff>
--- a/Jaguars-Jumps-Home-Data.xlsx
+++ b/Jaguars-Jumps-Home-Data.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Testables" sheetId="4" r:id="rId4"/>
     <sheet name="Plan" sheetId="5" r:id="rId5"/>
     <sheet name="Sessions" sheetId="6" r:id="rId6"/>
+    <sheet name="Calendar" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -2006,4 +2007,226 @@
     <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E12"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Event</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Location</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="B2" t="str">
+        <v>First Day of Winter Track</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Milestone</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-12-21</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Winter Break Begins</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2027-02-12</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Parent Meeting</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2027-02-20</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Spring Season Begins</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Milestone</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2027-02-22</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Final Reporting Deadline</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Deadline</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2027-03-22</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Spring Break</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2027-03-23</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Spring Break</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2027-03-24</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Spring Break</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2027-03-25</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Spring Break</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2027-03-26</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Spring Break</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2027-05-27</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Last Day of School</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Milestone</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>